<commit_message>
Caso 16 LavaYa: nombres reales de clientes, servicios y locales (mismas cifras)
</commit_message>
<xml_diff>
--- a/PMD1_15_Casos_Sinteticos/16_Lavanderia_PMD1.xlsx
+++ b/PMD1_15_Casos_Sinteticos/16_Lavanderia_PMD1.xlsx
@@ -19252,7 +19252,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Cliente 1</t>
+          <t>Ana Quispe Vargas</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -19272,7 +19272,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Cliente 2</t>
+          <t>Luis Rojas Paredes</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -19292,7 +19292,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Cliente 3</t>
+          <t>María Castillo Sayán</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -19312,7 +19312,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Cliente 4</t>
+          <t>Jorge Ramírez Castillo</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -19332,7 +19332,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Cliente 5</t>
+          <t>Rosa Paredes Ccori</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -19352,7 +19352,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Cliente 6</t>
+          <t>Carlos Delgado Quispe</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -19372,7 +19372,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Cliente 7</t>
+          <t>Lucía Valdivia Torres</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -19392,7 +19392,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Cliente 8</t>
+          <t>Miguel Flores Espinoza</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -19412,7 +19412,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Cliente 9 </t>
+          <t xml:space="preserve">  Carmen Mendoza Flores </t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -19432,7 +19432,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Cliente 10</t>
+          <t>José Torres Chávez</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -19452,7 +19452,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Cliente 11</t>
+          <t>Patricia Gutiérrez Delgado</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -19472,7 +19472,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Cliente 12</t>
+          <t>Diego Ccori Huamán</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -19492,7 +19492,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Cliente 13</t>
+          <t>Milagros Aguilar Ramírez</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -19512,7 +19512,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Cliente 14</t>
+          <t>Renzo Sayán Aguilar</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -19532,7 +19532,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Cliente 15</t>
+          <t>Gabriela Huamán Rojas</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -19552,7 +19552,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Cliente 16</t>
+          <t>Hugo Vargas Gutiérrez</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -19572,7 +19572,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Cliente 17</t>
+          <t>Fiorella Chávez Cárdenas</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -19592,7 +19592,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Cliente 18</t>
+          <t>César Salazar Mendoza</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -19612,7 +19612,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Cliente 19</t>
+          <t>Paola Espinoza Salazar</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -19632,7 +19632,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Cliente 20</t>
+          <t>Iván Cárdenas Valdivia</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -19652,7 +19652,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Cliente 21</t>
+          <t>Sofía Quispe Vargas</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -19672,7 +19672,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Cliente 22</t>
+          <t>Martín Rojas Paredes</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -19692,7 +19692,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Cliente 23</t>
+          <t>Ana Castillo Sayán</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -19712,7 +19712,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Cliente 24 </t>
+          <t xml:space="preserve">  Luis Ramírez Castillo </t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -19732,7 +19732,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Cliente 25</t>
+          <t>María Paredes Ccori</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -19752,7 +19752,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Cliente 26</t>
+          <t>Jorge Delgado Quispe</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -19772,7 +19772,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Cliente 27</t>
+          <t>Rosa Valdivia Torres</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -19792,7 +19792,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Cliente 28</t>
+          <t>Carlos Flores Espinoza</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -19812,7 +19812,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Cliente 29</t>
+          <t>Lucía Mendoza Flores</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -19832,7 +19832,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Cliente 30</t>
+          <t>Miguel Torres Chávez</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -19852,7 +19852,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Cliente 31</t>
+          <t>Carmen Gutiérrez Delgado</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -19872,7 +19872,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Cliente 32</t>
+          <t>José Ccori Huamán</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -19892,7 +19892,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Cliente 33</t>
+          <t>Patricia Aguilar Ramírez</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -19912,7 +19912,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Cliente 34</t>
+          <t>Diego Sayán Aguilar</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -19932,7 +19932,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Cliente 35</t>
+          <t>Milagros Huamán Rojas</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -19952,7 +19952,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Cliente 36</t>
+          <t>Renzo Vargas Gutiérrez</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -19972,7 +19972,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Cliente 37</t>
+          <t>Gabriela Chávez Cárdenas</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -19992,7 +19992,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Cliente 38</t>
+          <t>Hugo Salazar Mendoza</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -20012,7 +20012,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Cliente 39</t>
+          <t>Fiorella Espinoza Salazar</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -20032,7 +20032,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Cliente 40</t>
+          <t>César Cárdenas Valdivia</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -20052,7 +20052,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Cliente 41</t>
+          <t>Paola Quispe Vargas</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -20072,7 +20072,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Cliente 42</t>
+          <t>Iván Rojas Paredes</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -20092,7 +20092,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Cliente 43</t>
+          <t>Sofía Castillo Sayán</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -20112,7 +20112,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Cliente 44</t>
+          <t>Martín Ramírez Castillo</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -20132,7 +20132,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Cliente 45</t>
+          <t>Ana Paredes Ccori</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -20152,7 +20152,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Cliente 46</t>
+          <t>Luis Delgado Quispe</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -20172,7 +20172,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Cliente 47</t>
+          <t>María Valdivia Torres</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -20192,7 +20192,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Cliente 48</t>
+          <t>Jorge Flores Espinoza</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -20212,7 +20212,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Cliente 49</t>
+          <t>Rosa Mendoza Flores</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -20232,7 +20232,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Cliente 50</t>
+          <t>Carlos Torres Chávez</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -20252,7 +20252,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Cliente 51</t>
+          <t>Lucía Gutiérrez Delgado</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -20272,7 +20272,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Cliente 52</t>
+          <t>Miguel Ccori Huamán</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -20292,7 +20292,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Cliente 53</t>
+          <t>Carmen Aguilar Ramírez</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
@@ -20312,7 +20312,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Cliente 54</t>
+          <t>José Sayán Aguilar</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -20332,7 +20332,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Cliente 55</t>
+          <t>Patricia Huamán Rojas</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
@@ -20352,7 +20352,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Cliente 56</t>
+          <t>Diego Vargas Gutiérrez</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
@@ -20372,7 +20372,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Cliente 57</t>
+          <t>Milagros Chávez Cárdenas</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
@@ -20392,7 +20392,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Cliente 58</t>
+          <t>Renzo Salazar Mendoza</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
@@ -20412,7 +20412,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Cliente 59</t>
+          <t>Gabriela Espinoza Salazar</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
@@ -20432,7 +20432,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Cliente 60</t>
+          <t>Hugo Cárdenas Valdivia</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
@@ -20452,7 +20452,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Cliente 61</t>
+          <t>Fiorella Quispe Vargas</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
@@ -20472,7 +20472,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Cliente 62</t>
+          <t>César Rojas Paredes</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
@@ -20492,7 +20492,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Cliente 63</t>
+          <t>Paola Castillo Sayán</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
@@ -20512,7 +20512,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Cliente 64</t>
+          <t>Iván Ramírez Castillo</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
@@ -20532,7 +20532,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>Cliente 65</t>
+          <t>Sofía Paredes Ccori</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
@@ -20552,7 +20552,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>Cliente 66</t>
+          <t>Martín Delgado Quispe</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
@@ -20572,7 +20572,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>Cliente 67</t>
+          <t>Ana Valdivia Torres</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
@@ -20592,7 +20592,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>Cliente 68</t>
+          <t>Luis Flores Espinoza</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
@@ -20612,7 +20612,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Cliente 69 </t>
+          <t xml:space="preserve">  María Mendoza Flores </t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
@@ -20632,7 +20632,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>Cliente 70</t>
+          <t>Jorge Torres Chávez</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
@@ -20652,7 +20652,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>Cliente 71</t>
+          <t>Rosa Gutiérrez Delgado</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
@@ -20672,7 +20672,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>Cliente 72</t>
+          <t>Carlos Ccori Huamán</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
@@ -20692,7 +20692,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>Cliente 73</t>
+          <t>Lucía Aguilar Ramírez</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
@@ -20712,7 +20712,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>Cliente 74</t>
+          <t>Miguel Sayán Aguilar</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
@@ -20732,7 +20732,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>Cliente 75</t>
+          <t>Carmen Huamán Rojas</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
@@ -20752,7 +20752,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>Cliente 76</t>
+          <t>José Vargas Gutiérrez</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
@@ -20772,7 +20772,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>Cliente 77</t>
+          <t>Patricia Chávez Cárdenas</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
@@ -20792,7 +20792,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>Cliente 78</t>
+          <t>Diego Salazar Mendoza</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
@@ -20812,7 +20812,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>Cliente 79</t>
+          <t>Milagros Espinoza Salazar</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
@@ -20832,7 +20832,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>Cliente 80</t>
+          <t>Renzo Cárdenas Valdivia</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
@@ -20852,7 +20852,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>Cliente 81</t>
+          <t>Gabriela Quispe Vargas</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
@@ -20872,7 +20872,7 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>Cliente 82</t>
+          <t>Hugo Rojas Paredes</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
@@ -20892,7 +20892,7 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>Cliente 83</t>
+          <t>Fiorella Castillo Sayán</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
@@ -20912,7 +20912,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>Cliente 84</t>
+          <t>César Ramírez Castillo</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
@@ -20932,7 +20932,7 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>Cliente 85</t>
+          <t>Paola Paredes Ccori</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
@@ -20952,7 +20952,7 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>Cliente 86</t>
+          <t>Iván Delgado Quispe</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
@@ -20972,7 +20972,7 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Cliente 87 </t>
+          <t xml:space="preserve">  Sofía Valdivia Torres </t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
@@ -20992,7 +20992,7 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>Cliente 88</t>
+          <t>Martín Flores Espinoza</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
@@ -21012,7 +21012,7 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>Cliente 89</t>
+          <t>Ana Mendoza Flores</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
@@ -21032,7 +21032,7 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>Cliente 90</t>
+          <t>Luis Torres Chávez</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
@@ -21052,7 +21052,7 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>Cliente 91</t>
+          <t>María Gutiérrez Delgado</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
@@ -21072,7 +21072,7 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>Cliente 92</t>
+          <t>Jorge Ccori Huamán</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
@@ -21092,7 +21092,7 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>Cliente 93</t>
+          <t>Rosa Aguilar Ramírez</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
@@ -21112,7 +21112,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>Cliente 94</t>
+          <t>Carlos Sayán Aguilar</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
@@ -21132,7 +21132,7 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>Cliente 95</t>
+          <t>Lucía Huamán Rojas</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
@@ -21152,7 +21152,7 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>Cliente 96</t>
+          <t>Miguel Vargas Gutiérrez</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
@@ -21172,7 +21172,7 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>Cliente 97</t>
+          <t>Carmen Chávez Cárdenas</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
@@ -21192,7 +21192,7 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Cliente 98 </t>
+          <t xml:space="preserve">  José Salazar Mendoza </t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
@@ -21212,7 +21212,7 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>Cliente 99</t>
+          <t>Patricia Espinoza Salazar</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
@@ -21232,7 +21232,7 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>Cliente 100</t>
+          <t>Diego Cárdenas Valdivia</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
@@ -21252,7 +21252,7 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>Cliente 101</t>
+          <t>Milagros Quispe Vargas</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
@@ -21272,7 +21272,7 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>Cliente 102</t>
+          <t>Renzo Rojas Paredes</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
@@ -21292,7 +21292,7 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>Cliente 103</t>
+          <t>Gabriela Castillo Sayán</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
@@ -21312,7 +21312,7 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>Cliente 104</t>
+          <t>Hugo Ramírez Castillo</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
@@ -21332,7 +21332,7 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>Cliente 105</t>
+          <t>Fiorella Paredes Ccori</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
@@ -21352,7 +21352,7 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Cliente 106 </t>
+          <t xml:space="preserve">  César Delgado Quispe </t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
@@ -21372,7 +21372,7 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>Cliente 107</t>
+          <t>Paola Valdivia Torres</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
@@ -21392,7 +21392,7 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>Cliente 108</t>
+          <t>Iván Flores Espinoza</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
@@ -21412,7 +21412,7 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>Cliente 109</t>
+          <t>Sofía Mendoza Flores</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
@@ -21432,7 +21432,7 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>Cliente 110</t>
+          <t>Martín Torres Chávez</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
@@ -21499,7 +21499,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>lavado por kilo 1</t>
+          <t>Lavado por kilo estándar</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -21519,7 +21519,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>lavado al seco 2</t>
+          <t>Lavado al seco de terno</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -21539,7 +21539,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>planchado 3</t>
+          <t>Planchado de camisas</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -21559,7 +21559,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>edredones 4</t>
+          <t>Edredón individual</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -21579,7 +21579,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>zapatillas 5</t>
+          <t>Limpieza de zapatillas de lona</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -21599,7 +21599,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>lavado por kilo 6</t>
+          <t>Lavado por kilo express</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -21619,7 +21619,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>lavado al seco 7</t>
+          <t>Lavado al seco de vestido</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -21639,7 +21639,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>planchado 8</t>
+          <t>Planchado de pantalones</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -21659,7 +21659,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>edredones 9</t>
+          <t>Edredón 2 plazas</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -21679,7 +21679,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>zapatillas 10</t>
+          <t>Limpieza de zapatillas de cuero</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -21699,7 +21699,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>lavado por kilo 11</t>
+          <t>Lavado por kilo ropa de cama</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -21719,7 +21719,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>lavado al seco 12</t>
+          <t>Lavado al seco de abrigo</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -21739,7 +21739,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>planchado 13</t>
+          <t>Planchado de manteles</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -21759,7 +21759,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>edredones 14</t>
+          <t>Edredón king</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -21779,7 +21779,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>zapatillas 15</t>
+          <t>Limpieza de zapatillas deportivas</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -21799,7 +21799,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>lavado por kilo 16</t>
+          <t>Lavado por kilo ropa deportiva</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -21819,7 +21819,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>lavado al seco 17</t>
+          <t>Lavado al seco de casaca de cuero</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -21839,7 +21839,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>planchado 18</t>
+          <t>Planchado de cortinas</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -21901,7 +21901,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Lavanderia sede 1</t>
+          <t>LavaYa Cercado de Lima</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -21918,7 +21918,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Lavanderia sede 2</t>
+          <t>LavaYa Los Olivos</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -21935,7 +21935,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Lavanderia sede 3</t>
+          <t>LavaYa Surco</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -21952,7 +21952,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Lavanderia sede 4</t>
+          <t>LavaYa La Molina</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -21969,7 +21969,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Lavanderia sede 5</t>
+          <t>LavaYa Trujillo Centro</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">

</xml_diff>